<commit_message>
Refine CDA RTO_PQ_PQ to FHIR Ratio mapping details
Updated the mapping details for CDA RTO_PQ_PQ to FHIR Ratio, including changes to URLs, source and target definitions, and display values. dbe2fe3bd2421adafd2bf3532163c3f950a90392
</commit_message>
<xml_diff>
--- a/traitement-erreur/ig/CdaRTO-PQ-PQToRatioConceptMap.xlsx
+++ b/traitement-erreur/ig/CdaRTO-PQ-PQToRatioConceptMap.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>Property</t>
   </si>
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/DataTypes/CdaRTOPQPQToFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/mappingcdafhir/ConceptMap/CdaRTO-PQ-PQToRatioConceptMap</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-22T13:44:26+00:00</t>
+    <t>2026-07-22T13:54:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -105,7 +105,7 @@
     <t>Target</t>
   </si>
   <si>
-    <t>http://hl7.org/cda/stds/core/StructureDefinition/RTO_PQ_PQ</t>
+    <t>http://hl7.org/cda/stds/core/StructureDefinition/RTO-PQ-PQ|2.0.0-sd</t>
   </si>
   <si>
     <t/>
@@ -117,16 +117,28 @@
     <t>RTO_PQ_PQ.numerator</t>
   </si>
   <si>
+    <t>Numerator</t>
+  </si>
+  <si>
     <t>related-to</t>
   </si>
   <si>
     <t>Ratio.numerator</t>
   </si>
   <si>
+    <t>Numerator value</t>
+  </si>
+  <si>
     <t>RTO_PQ_PQ.denominator</t>
   </si>
   <si>
+    <t>Denominator</t>
+  </si>
+  <si>
     <t>Ratio.denominator</t>
+  </si>
+  <si>
+    <t>Denominator value</t>
   </si>
 </sst>
 </file>
@@ -424,33 +436,33 @@
         <v>33</v>
       </c>
       <c r="B3" t="s" s="2">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="2">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s" s="2">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>